<commit_message>
scan: seg4 2026-06-12 17:08 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq5_2026-06-12.xlsx
+++ b/output/full_scan/batch_seq5_2026-06-12.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O80"/>
+  <dimension ref="A1:O82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -792,21 +792,21 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>5515</v>
+        <v>4807</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>建國</t>
+          <t>日成-KY</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>721.2226865452039</v>
+        <v>728.6979283415221</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -817,16 +817,16 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>72.41484482861502</v>
+        <v>78.87395670961052</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>21.92526496100084</v>
+        <v>60.97670294712506</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>1.122268654520396</v>
+        <v>0.8697928341522182</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L7" s="2" t="n">
         <v>0</v>
@@ -835,31 +835,31 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.2858163417093992</v>
+        <v>0.8098063286947532</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, adx_trending, obv_uptrend, bb_squeeze_breakout, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>4306</v>
+        <v>5515</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>炎洲</t>
+          <t>建國</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>711.4653144466905</v>
+        <v>721.2226865452039</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>16.1</v>
+        <v>44</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -870,13 +870,13 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>85.80018825890907</v>
+        <v>72.41484482861502</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>42.15380473970585</v>
+        <v>21.92526496100084</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>2.14653144466905</v>
+        <v>1.122268654520396</v>
       </c>
       <c r="K8" s="2" t="n">
         <v>0</v>
@@ -888,31 +888,31 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.1706262014314863</v>
+        <v>0.2858163417093992</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, adx_trending, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, adx_trending, obv_uptrend, bb_squeeze_breakout, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>4739</v>
+        <v>4306</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>康普</t>
+          <t>炎洲</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
         <v/>
       </c>
       <c r="D9" s="2" t="n">
-        <v>704.1493567368813</v>
+        <v>711.4653144466905</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>121.5</v>
+        <v>16.1</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -923,13 +923,13 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>64.04236510170628</v>
+        <v>85.80018825890907</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>31.66664098125847</v>
+        <v>42.15380473970585</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>0.914935673688124</v>
+        <v>2.14653144466905</v>
       </c>
       <c r="K9" s="2" t="n">
         <v>0</v>
@@ -941,31 +941,31 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>1.134874832793771</v>
+        <v>0.1706262014314863</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, adx_trending, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>6156</v>
+        <v>4739</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>松上</t>
+          <t>康普</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>690.1591685477355</v>
+        <v>704.1493567368813</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>20.55</v>
+        <v>121.5</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -976,13 +976,13 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>60.94274561283981</v>
+        <v>64.04236510170628</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>13.47732478413917</v>
+        <v>31.66664098125847</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>3.515916854773552</v>
+        <v>0.914935673688124</v>
       </c>
       <c r="K10" s="2" t="n">
         <v>0</v>
@@ -994,31 +994,31 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.1866887489174329</v>
+        <v>1.134874832793771</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, volume_break, rsi_strong, breakout_20d, market_above_ma60, obv_uptrend, bb_squeeze_breakout, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>6024</v>
+        <v>6116</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>群益期</t>
+          <t>彩晶</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
         <v/>
       </c>
       <c r="D11" s="2" t="n">
-        <v>678.7437458119672</v>
+        <v>701.8311289590233</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>61.5</v>
+        <v>15.6</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -1029,16 +1029,16 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>71.48599785037244</v>
+        <v>54.3264977807434</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>27.22838088859302</v>
+        <v>40.36346779290179</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>0.8743745811967143</v>
+        <v>0.1831128959023278</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L11" s="2" t="n">
         <v>0</v>
@@ -1047,31 +1047,31 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.3035027811658151</v>
+        <v>-0.4855556943652317</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>5534</v>
+        <v>6156</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>長虹</t>
+          <t>松上</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
         <v/>
       </c>
       <c r="D12" s="2" t="n">
-        <v>670.6661495311389</v>
+        <v>690.1591685477355</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>83.40000000000001</v>
+        <v>20.55</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -1082,13 +1082,13 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>69.86792683166777</v>
+        <v>60.94274561283981</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>31.00749278249691</v>
+        <v>13.47732478413917</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>1.566614953113895</v>
+        <v>3.515916854773552</v>
       </c>
       <c r="K12" s="2" t="n">
         <v>0</v>
@@ -1100,31 +1100,31 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>1.08881519327225</v>
+        <v>0.1866887489174329</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, volume_break, rsi_strong, breakout_20d, market_above_ma60, obv_uptrend, bb_squeeze_breakout, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>5880</v>
+        <v>6024</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>合庫金</t>
+          <t>群益期</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>664.9119214580296</v>
+        <v>678.7437458119672</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>24.05</v>
+        <v>61.5</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -1135,13 +1135,13 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>66.94831592516239</v>
+        <v>71.48599785037244</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>29.83008876309358</v>
+        <v>27.22838088859302</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>0.9911921458029664</v>
+        <v>0.8743745811967143</v>
       </c>
       <c r="K13" s="2" t="n">
         <v>0</v>
@@ -1153,31 +1153,31 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0.1326436317656008</v>
+        <v>0.3035027811658151</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>5871</v>
+        <v>5534</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>中租-KY</t>
+          <t>長虹</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
         <v/>
       </c>
       <c r="D14" s="2" t="n">
-        <v>651.8740960686548</v>
+        <v>670.6661495311389</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>121.5</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -1188,13 +1188,13 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>64.43053422146244</v>
+        <v>69.86792683166777</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>21.67158100638257</v>
+        <v>31.00749278249691</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>0.6874096068654809</v>
+        <v>1.566614953113895</v>
       </c>
       <c r="K14" s="2" t="n">
         <v>0</v>
@@ -1206,31 +1206,31 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>1.263013932495586</v>
+        <v>1.08881519327225</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>5288</v>
+        <v>5880</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>豐祥-KY</t>
+          <t>合庫金</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v/>
       </c>
       <c r="D15" s="2" t="n">
-        <v>651.6436885278916</v>
+        <v>664.9119214580296</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>190.5</v>
+        <v>24.05</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1241,13 +1241,13 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>80.09878817280384</v>
+        <v>66.94831592516239</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>24.81852206844126</v>
+        <v>29.83008876309358</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>2.164368852789166</v>
+        <v>0.9911921458029664</v>
       </c>
       <c r="K15" s="2" t="n">
         <v>0</v>
@@ -1259,31 +1259,31 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>3.748124945675535</v>
+        <v>0.1326436317656008</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>6138</v>
+        <v>5871</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>茂達</t>
+          <t>中租-KY</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>649.2717677513147</v>
+        <v>651.8740960686548</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>313</v>
+        <v>121.5</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -1294,13 +1294,13 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>52.63591287410598</v>
+        <v>64.43053422146244</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>30.53038079991035</v>
+        <v>21.67158100638257</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>0.4271767751314706</v>
+        <v>0.6874096068654809</v>
       </c>
       <c r="K16" s="2" t="n">
         <v>0</v>
@@ -1312,31 +1312,31 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>-7.25121136675785</v>
+        <v>1.263013932495586</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>5607</v>
+        <v>5288</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>遠雄港</t>
+          <t>豐祥-KY</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
         <v/>
       </c>
       <c r="D17" s="2" t="n">
-        <v>646.274127638462</v>
+        <v>651.6436885278916</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>52.5</v>
+        <v>190.5</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1347,13 +1347,13 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>59.72608459681776</v>
+        <v>80.09878817280384</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>26.77883867901114</v>
+        <v>24.81852206844126</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>1.127412763846202</v>
+        <v>2.164368852789166</v>
       </c>
       <c r="K17" s="2" t="n">
         <v>0</v>
@@ -1365,31 +1365,31 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.1063040497416107</v>
+        <v>3.748124945675535</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>5522</v>
+        <v>6138</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>遠雄</t>
+          <t>茂達</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
         <v/>
       </c>
       <c r="D18" s="2" t="n">
-        <v>645.2788973444104</v>
+        <v>649.2717677513147</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>80</v>
+        <v>313</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1400,13 +1400,13 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>66.00681310805911</v>
+        <v>52.63591287410598</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>30.57905666353019</v>
+        <v>30.53038079991035</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>1.027889734441042</v>
+        <v>0.4271767751314706</v>
       </c>
       <c r="K18" s="2" t="n">
         <v>0</v>
@@ -1418,31 +1418,31 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>0.7663898276494727</v>
+        <v>-7.25121136675785</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>4540</v>
+        <v>5607</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>全球傳動</t>
+          <t>遠雄港</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>632.0312418421041</v>
+        <v>646.274127638462</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>61.5</v>
+        <v>52.5</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -1453,13 +1453,13 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>42.57644890434555</v>
+        <v>59.72608459681776</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>23.50658728501962</v>
+        <v>26.77883867901114</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>0.203124184210409</v>
+        <v>1.127412763846202</v>
       </c>
       <c r="K19" s="2" t="n">
         <v>0</v>
@@ -1471,31 +1471,31 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>-1.758929211844332</v>
+        <v>0.1063040497416107</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>4590</v>
+        <v>5522</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>富田-創</t>
+          <t>遠雄</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
         <v/>
       </c>
       <c r="D20" s="2" t="n">
-        <v>630.0219418760104</v>
+        <v>645.2788973444104</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>76.09999999999999</v>
+        <v>80</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1506,13 +1506,13 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>57.20854745525005</v>
+        <v>66.00681310805911</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>9.114978911194671</v>
+        <v>30.57905666353019</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>1.502194187601041</v>
+        <v>1.027889734441042</v>
       </c>
       <c r="K20" s="2" t="n">
         <v>0</v>
@@ -1524,31 +1524,31 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0.4163277367384285</v>
+        <v>0.7663898276494727</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, volume_break, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, obv_uptrend, bb_squeeze_breakout, breakout_volume_confirm</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>4552</v>
+        <v>4540</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>力達-KY</t>
+          <t>全球傳動</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
         <v/>
       </c>
       <c r="D21" s="2" t="n">
-        <v>615.9183249611641</v>
+        <v>632.0312418421041</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21.3</v>
+        <v>61.5</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1559,13 +1559,13 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>68.80019328037645</v>
+        <v>42.57644890434555</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>28.95456620673193</v>
+        <v>23.50658728501962</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>0.5918324961164128</v>
+        <v>0.203124184210409</v>
       </c>
       <c r="K21" s="2" t="n">
         <v>0</v>
@@ -1577,31 +1577,31 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>0.1358721978772211</v>
+        <v>-1.758929211844332</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>5706</v>
+        <v>4590</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>鳳凰</t>
+          <t>富田-創</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>614.6768671322377</v>
+        <v>630.0219418760104</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>53</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -1612,13 +1612,13 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>60.86055364841405</v>
+        <v>57.20854745525005</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>20.83196793772564</v>
+        <v>9.114978911194671</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>1.467686713223772</v>
+        <v>1.502194187601041</v>
       </c>
       <c r="K22" s="2" t="n">
         <v>0</v>
@@ -1630,31 +1630,31 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.1791063717421707</v>
+        <v>0.4163277367384285</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, volume_break, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, obv_uptrend, bb_squeeze_breakout, breakout_volume_confirm</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>6134</v>
+        <v>4552</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>萬旭</t>
+          <t>力達-KY</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
         <v/>
       </c>
       <c r="D23" s="2" t="n">
-        <v>609.8065294047511</v>
+        <v>615.9183249611641</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>35.5</v>
+        <v>21.3</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -1665,13 +1665,13 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>56.87331748090049</v>
+        <v>68.80019328037645</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>16.63701937318327</v>
+        <v>28.95456620673193</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>1.480652940475111</v>
+        <v>0.5918324961164128</v>
       </c>
       <c r="K23" s="2" t="n">
         <v>0</v>
@@ -1683,31 +1683,31 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>-0.1026859230711998</v>
+        <v>0.1358721978772211</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>6147</v>
+        <v>5706</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>頎邦</t>
+          <t>鳳凰</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>580.5915877400934</v>
+        <v>614.6768671322377</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>224</v>
+        <v>53</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1718,13 +1718,13 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>48.56673813302986</v>
+        <v>60.86055364841405</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>42.7302447584561</v>
+        <v>20.83196793772564</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>0.5591587740093359</v>
+        <v>1.467686713223772</v>
       </c>
       <c r="K24" s="2" t="n">
         <v>0</v>
@@ -1736,31 +1736,31 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>-9.968600529177866</v>
+        <v>0.1791063717421707</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>4526</v>
+        <v>6134</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>東台</t>
+          <t>萬旭</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>574.2659520940425</v>
+        <v>609.8065294047511</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>38.8</v>
+        <v>35.5</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1771,13 +1771,13 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>49.02662036092632</v>
+        <v>56.87331748090049</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>31.54989817504964</v>
+        <v>16.63701937318327</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>0.4265952094042546</v>
+        <v>1.480652940475111</v>
       </c>
       <c r="K25" s="2" t="n">
         <v>0</v>
@@ -1789,31 +1789,31 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>-0.5188683101626155</v>
+        <v>-0.1026859230711998</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>6161</v>
+        <v>6147</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>捷波</t>
+          <t>頎邦</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>567.6966915577181</v>
+        <v>580.5915877400934</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>53.7</v>
+        <v>224</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1824,13 +1824,13 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>53.10617725766288</v>
+        <v>48.56673813302986</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>29.48362148949524</v>
+        <v>42.7302447584561</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>0.2696691557718075</v>
+        <v>0.5591587740093359</v>
       </c>
       <c r="K26" s="2" t="n">
         <v>0</v>
@@ -1842,31 +1842,31 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>-0.924938631354168</v>
+        <v>-9.968600529177866</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>6154</v>
+        <v>4526</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>順發</t>
+          <t>東台</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>564.7504469276257</v>
+        <v>574.2659520940425</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>14</v>
+        <v>38.8</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1877,13 +1877,13 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>67.22459775592137</v>
+        <v>49.02662036092632</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>33.9232700398535</v>
+        <v>31.54989817504964</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>0.9750446927625688</v>
+        <v>0.4265952094042546</v>
       </c>
       <c r="K27" s="2" t="n">
         <v>0</v>
@@ -1895,31 +1895,31 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.0511527927926891</v>
+        <v>-0.5188683101626155</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>4771</v>
+        <v>6161</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>望隼</t>
+          <t>捷波</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>562.956548407634</v>
+        <v>567.6966915577181</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>189.5</v>
+        <v>53.7</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1930,13 +1930,13 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>45.58145222897669</v>
+        <v>53.10617725766288</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>20.43245456894479</v>
+        <v>29.48362148949524</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>0.2956548407634033</v>
+        <v>0.2696691557718075</v>
       </c>
       <c r="K28" s="2" t="n">
         <v>0</v>
@@ -1948,31 +1948,31 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>-1.332154396817808</v>
+        <v>-0.924938631354168</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>5533</v>
+        <v>6154</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>皇鼎</t>
+          <t>順發</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>562.4613228904702</v>
+        <v>564.7504469276257</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>14.15</v>
+        <v>14</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1983,13 +1983,13 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>56.12861551507454</v>
+        <v>67.22459775592137</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>23.18474650808605</v>
+        <v>33.9232700398535</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>0.746132289047019</v>
+        <v>0.9750446927625688</v>
       </c>
       <c r="K29" s="2" t="n">
         <v>0</v>
@@ -2001,31 +2001,31 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.0338434455570572</v>
+        <v>0.0511527927926891</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, adx_trending, bb_squeeze_breakout, mfi_strong</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>6163</v>
+        <v>4771</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>華電網</t>
+          <t>望隼</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>549.8353726938251</v>
+        <v>562.956548407634</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>51.3</v>
+        <v>189.5</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -2036,13 +2036,13 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>44.99735080994159</v>
+        <v>45.58145222897669</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>16.08645128461654</v>
+        <v>20.43245456894479</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>0.4835372693825023</v>
+        <v>0.2956548407634033</v>
       </c>
       <c r="K30" s="2" t="n">
         <v>0</v>
@@ -2054,31 +2054,31 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>0.038416310848961</v>
+        <v>-1.332154396817808</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>4763</v>
+        <v>5533</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>材料*-KY</t>
+          <t>皇鼎</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>546.3376671323173</v>
+        <v>562.4613228904702</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>44.45</v>
+        <v>14.15</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -2089,13 +2089,13 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>55.38804587476507</v>
+        <v>56.12861551507454</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>16.55906620273338</v>
+        <v>23.18474650808605</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>0.6337667132317224</v>
+        <v>0.746132289047019</v>
       </c>
       <c r="K31" s="2" t="n">
         <v>0</v>
@@ -2107,31 +2107,31 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.2711607111584255</v>
+        <v>0.0338434455570572</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, adx_trending, bb_squeeze_breakout, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>5876</v>
+        <v>6163</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>上海商銀</t>
+          <t>華電網</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>540.9320017021437</v>
+        <v>549.8353726938251</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>42.5</v>
+        <v>51.3</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2142,13 +2142,13 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>65.72164553116424</v>
+        <v>44.99735080994159</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>24.75880177185082</v>
+        <v>16.08645128461654</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>0.5932001702143697</v>
+        <v>0.4835372693825023</v>
       </c>
       <c r="K32" s="2" t="n">
         <v>0</v>
@@ -2160,31 +2160,31 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.2438104614392837</v>
+        <v>0.038416310848961</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>4438</v>
+        <v>4763</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>廣越</t>
+          <t>材料*-KY</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>538.3971266269264</v>
+        <v>546.3376671323173</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>61.3</v>
+        <v>44.45</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,13 +2195,13 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>55.178104893351</v>
+        <v>55.38804587476507</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>34.32352573717261</v>
+        <v>16.55906620273338</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>0.3397126626926355</v>
+        <v>0.6337667132317224</v>
       </c>
       <c r="K33" s="2" t="n">
         <v>0</v>
@@ -2213,31 +2213,31 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.0546381674837151</v>
+        <v>0.2711607111584255</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>6160</v>
+        <v>5876</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>欣技</t>
+          <t>上海商銀</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>514.5766219033492</v>
+        <v>540.9320017021437</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>16.6</v>
+        <v>42.5</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2248,13 +2248,13 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>49.20469353948581</v>
+        <v>65.72164553116424</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>23.4651235663377</v>
+        <v>24.75880177185082</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>0.4576621903349186</v>
+        <v>0.5932001702143697</v>
       </c>
       <c r="K34" s="2" t="n">
         <v>0</v>
@@ -2266,31 +2266,31 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>-0.0704764380931923</v>
+        <v>0.2438104614392837</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>6150</v>
+        <v>4438</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>撼訊</t>
+          <t>廣越</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>514.3813833823358</v>
+        <v>538.3971266269264</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>64</v>
+        <v>61.3</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -2301,13 +2301,13 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>46.54470597572633</v>
+        <v>55.178104893351</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>30.47200475009579</v>
+        <v>34.32352573717261</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>0.4381383382335825</v>
+        <v>0.3397126626926355</v>
       </c>
       <c r="K35" s="2" t="n">
         <v>0</v>
@@ -2319,31 +2319,31 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>-1.223768221994706</v>
+        <v>0.0546381674837151</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>4576</v>
+        <v>6160</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>大銀微系統</t>
+          <t>欣技</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>513.80673772425</v>
+        <v>514.5766219033492</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>202</v>
+        <v>16.6</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -2354,13 +2354,13 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>39.70785523710782</v>
+        <v>49.20469353948581</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>29.51934247063729</v>
+        <v>23.4651235663377</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>0.3806737724249932</v>
+        <v>0.4576621903349186</v>
       </c>
       <c r="K36" s="2" t="n">
         <v>0</v>
@@ -2372,31 +2372,31 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-8.893545070782212</v>
+        <v>-0.0704764380931923</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>4551</v>
+        <v>6150</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>智伸科</t>
+          <t>撼訊</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>509.4631667907052</v>
+        <v>514.3813833823358</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>152</v>
+        <v>64</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2407,13 +2407,13 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>55.87005955445518</v>
+        <v>46.54470597572633</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>23.58684024085672</v>
+        <v>30.47200475009579</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>1.446316679070517</v>
+        <v>0.4381383382335825</v>
       </c>
       <c r="K37" s="2" t="n">
         <v>0</v>
@@ -2425,31 +2425,31 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-1.391252052779506</v>
+        <v>-1.223768221994706</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>4532</v>
+        <v>4576</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>瑞智</t>
+          <t>大銀微系統</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>508.2288948244481</v>
+        <v>513.80673772425</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>24.45</v>
+        <v>202</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2460,13 +2460,13 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>54.6569626602124</v>
+        <v>39.70785523710782</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>21.49973080472621</v>
+        <v>29.51934247063729</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>0.8228894824448046</v>
+        <v>0.3806737724249932</v>
       </c>
       <c r="K38" s="2" t="n">
         <v>0</v>
@@ -2478,31 +2478,31 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.0539705573638513</v>
+        <v>-8.893545070782212</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>5284</v>
+        <v>4551</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>jpp-KY</t>
+          <t>智伸科</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>503.5638573370229</v>
+        <v>509.4631667907052</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>364</v>
+        <v>152</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2513,13 +2513,13 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>42.26154119614923</v>
+        <v>55.87005955445518</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>33.8196459817527</v>
+        <v>23.58684024085672</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>0.3563857337022847</v>
+        <v>1.446316679070517</v>
       </c>
       <c r="K39" s="2" t="n">
         <v>0</v>
@@ -2531,31 +2531,31 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-10.89784437541782</v>
+        <v>-1.391252052779506</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>4764</v>
+        <v>4532</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>雙鍵</t>
+          <t>瑞智</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>501.6565049219275</v>
+        <v>508.2288948244481</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>263</v>
+        <v>24.45</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2566,13 +2566,13 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>42.49143281139633</v>
+        <v>54.6569626602124</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>24.32403480522624</v>
+        <v>21.49973080472621</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>0.6656504921927479</v>
+        <v>0.8228894824448046</v>
       </c>
       <c r="K40" s="2" t="n">
         <v>0</v>
@@ -2584,31 +2584,31 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>-9.936137197988836</v>
+        <v>0.0539705573638513</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>5608</v>
+        <v>5284</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>四維航</t>
+          <t>jpp-KY</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>501.0786991239698</v>
+        <v>503.5638573370229</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>15.1</v>
+        <v>364</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2619,13 +2619,13 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>53.27545012169955</v>
+        <v>42.26154119614923</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>17.83013829832194</v>
+        <v>33.8196459817527</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>1.107869912396978</v>
+        <v>0.3563857337022847</v>
       </c>
       <c r="K41" s="2" t="n">
         <v>0</v>
@@ -2637,31 +2637,31 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.0962238563934984</v>
+        <v>-10.89784437541782</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>breakout_20d, market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>6151</v>
+        <v>4764</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>晉倫</t>
+          <t>雙鍵</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>494.3010161504799</v>
+        <v>501.6565049219275</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>42.25</v>
+        <v>263</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2672,13 +2672,13 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>50.47051440175981</v>
+        <v>42.49143281139633</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>29.42579529398537</v>
+        <v>24.32403480522624</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.4301016150479907</v>
+        <v>0.6656504921927479</v>
       </c>
       <c r="K42" s="2" t="n">
         <v>0</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-0.7758281464147181</v>
+        <v>-9.936137197988836</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2700,21 +2700,21 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>4571</v>
+        <v>5608</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>鈞興-KY</t>
+          <t>四維航</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>491.9327501346883</v>
+        <v>501.0786991239698</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>181</v>
+        <v>15.1</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2725,13 +2725,13 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>40.2176587302068</v>
+        <v>53.27545012169955</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>27.91477239412865</v>
+        <v>17.83013829832194</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.193275013468833</v>
+        <v>1.107869912396978</v>
       </c>
       <c r="K43" s="2" t="n">
         <v>0</v>
@@ -2743,31 +2743,31 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-5.167156155183476</v>
+        <v>0.0962238563934984</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>breakout_20d, market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>4766</v>
+        <v>6151</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>南寶</t>
+          <t>晉倫</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>482.2748399532234</v>
+        <v>494.3010161504799</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>369.5</v>
+        <v>42.25</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,13 +2778,13 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>51.90326054770344</v>
+        <v>50.47051440175981</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>20.69535702202758</v>
+        <v>29.42579529398537</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.7274839953223392</v>
+        <v>0.4301016150479907</v>
       </c>
       <c r="K44" s="2" t="n">
         <v>0</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-1.066181100628859</v>
+        <v>-0.7758281464147181</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2806,21 +2806,21 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>4722</v>
+        <v>4571</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>國精化</t>
+          <t>鈞興-KY</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>457.1577539625247</v>
+        <v>491.9327501346883</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>226.5</v>
+        <v>181</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,13 +2831,13 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>43.21244415248516</v>
+        <v>40.2176587302068</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>34.72822445618091</v>
+        <v>27.91477239412865</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>0.7157753962524703</v>
+        <v>0.193275013468833</v>
       </c>
       <c r="K45" s="2" t="n">
         <v>0</v>
@@ -2849,31 +2849,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-9.973818307947893</v>
+        <v>-5.167156155183476</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>5283</v>
+        <v>4766</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>禾聯碩</t>
+          <t>南寶</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>423.3832907302466</v>
+        <v>482.2748399532234</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>52.8</v>
+        <v>369.5</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,13 +2884,13 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>51.89472926324697</v>
+        <v>51.90326054770344</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>28.60115222852542</v>
+        <v>20.69535702202758</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0.8383290730246669</v>
+        <v>0.7274839953223392</v>
       </c>
       <c r="K46" s="2" t="n">
         <v>0</v>
@@ -2902,31 +2902,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.0732836356062205</v>
+        <v>-1.066181100628859</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>4572</v>
+        <v>4722</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>駐龍</t>
+          <t>國精化</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>419.98176758656</v>
+        <v>457.1577539625247</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>146.5</v>
+        <v>226.5</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,13 +2937,13 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>52.6829374225024</v>
+        <v>43.21244415248516</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>15.90491416473165</v>
+        <v>34.72822445618091</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.4981767586559995</v>
+        <v>0.7157753962524703</v>
       </c>
       <c r="K47" s="2" t="n">
         <v>0</v>
@@ -2955,31 +2955,31 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-0.0110195295631874</v>
+        <v>-9.973818307947893</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>6146</v>
+        <v>5283</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>耕興</t>
+          <t>禾聯碩</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>410.374128286865</v>
+        <v>423.3832907302466</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>196.5</v>
+        <v>52.8</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,13 +2990,13 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>34.42288300657671</v>
+        <v>51.89472926324697</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>23.94704397734914</v>
+        <v>28.60115222852542</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.5374128286864998</v>
+        <v>0.8383290730246669</v>
       </c>
       <c r="K48" s="2" t="n">
         <v>0</v>
@@ -3008,31 +3008,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-3.264577896901289</v>
+        <v>0.0732836356062205</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>4583</v>
+        <v>4572</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>台灣精銳</t>
+          <t>駐龍</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>399.0331525499705</v>
+        <v>419.98176758656</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>618</v>
+        <v>146.5</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,13 +3043,13 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>30.51596390758378</v>
+        <v>52.6829374225024</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>23.43308385761656</v>
+        <v>15.90491416473165</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.4033152549970494</v>
+        <v>0.4981767586559995</v>
       </c>
       <c r="K49" s="2" t="n">
         <v>0</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-10.07224136430187</v>
+        <v>-0.0110195295631874</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>4720</v>
+        <v>6146</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>德淵</t>
+          <t>耕興</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>397.5845593113453</v>
+        <v>410.374128286865</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>23.75</v>
+        <v>196.5</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,13 +3096,13 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>44.35533474980614</v>
+        <v>34.42288300657671</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>26.20410049372494</v>
+        <v>23.94704397734914</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.2584559311345359</v>
+        <v>0.5374128286864998</v>
       </c>
       <c r="K50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-0.4561767206110738</v>
+        <v>-3.264577896901289</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>4190</v>
+        <v>4583</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>佐登-KY</t>
+          <t>台灣精銳</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>384.7716815172797</v>
+        <v>399.0331525499705</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>24.9</v>
+        <v>618</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,13 +3149,13 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>48.98360023765276</v>
+        <v>30.51596390758378</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>35.65717014941538</v>
+        <v>23.43308385761656</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.4771681517279719</v>
+        <v>0.4033152549970494</v>
       </c>
       <c r="K51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.0782318404858611</v>
+        <v>-10.07224136430187</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>4414</v>
+        <v>4720</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>如興</t>
+          <t>德淵</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>383.44496987676</v>
+        <v>397.5845593113453</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>8.43</v>
+        <v>23.75</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,13 +3202,13 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>42.76385457042957</v>
+        <v>44.35533474980614</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>27.74456322449394</v>
+        <v>26.20410049372494</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.8444969876760019</v>
+        <v>0.2584559311345359</v>
       </c>
       <c r="K52" s="2" t="n">
         <v>0</v>
@@ -3220,31 +3220,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.1336819164384629</v>
+        <v>-0.4561767206110738</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>4566</v>
+        <v>4190</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>時碩工業</t>
+          <t>佐登-KY</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>382.6040252124653</v>
+        <v>384.7716815172797</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>63.2</v>
+        <v>24.9</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,13 +3255,13 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>45.90844489648742</v>
+        <v>48.98360023765276</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>14.63513510167739</v>
+        <v>35.65717014941538</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.7604025212465264</v>
+        <v>0.4771681517279719</v>
       </c>
       <c r="K53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-0.571406368507118</v>
+        <v>0.0782318404858611</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>5531</v>
+        <v>4414</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>鄉林</t>
+          <t>如興</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>380.8494245271468</v>
+        <v>383.44496987676</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>8.15</v>
+        <v>8.43</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>52.24769061786547</v>
+        <v>42.76385457042957</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>29.94618955688911</v>
+        <v>27.74456322449394</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.584942452714677</v>
+        <v>0.8444969876760019</v>
       </c>
       <c r="K54" s="2" t="n">
         <v>0</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.0781016706339439</v>
+        <v>0.1336819164384629</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3336,21 +3336,21 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>5525</v>
+        <v>4566</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>順天</t>
+          <t>時碩工業</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>379.9007307898736</v>
+        <v>382.6040252124653</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>22.3</v>
+        <v>63.2</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,13 +3361,13 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>49.38608703467234</v>
+        <v>45.90844489648742</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>32.42467569093063</v>
+        <v>14.63513510167739</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.4900730789873567</v>
+        <v>0.7604025212465264</v>
       </c>
       <c r="K55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.1590350425416684</v>
+        <v>-0.571406368507118</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>5538</v>
+        <v>5531</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>東明-KY</t>
+          <t>鄉林</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>374.2403813201082</v>
+        <v>380.8494245271468</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>32.45</v>
+        <v>8.15</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,13 +3414,13 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>43.37380752633383</v>
+        <v>52.24769061786547</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>32.84678507059154</v>
+        <v>29.94618955688911</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.4240381320108234</v>
+        <v>0.584942452714677</v>
       </c>
       <c r="K56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-0.50265201916005</v>
+        <v>0.0781016706339439</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>4930</v>
+        <v>5525</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>燦星網</t>
+          <t>順天</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>359.7198418646074</v>
+        <v>379.9007307898736</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>17.35</v>
+        <v>22.3</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,13 +3467,13 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>43.7333892054443</v>
+        <v>49.38608703467234</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>34.25901702495012</v>
+        <v>32.42467569093063</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.4719841864607431</v>
+        <v>0.4900730789873567</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.0277719202176923</v>
+        <v>0.1590350425416684</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3495,21 +3495,21 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>4562</v>
+        <v>5538</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>穎漢</t>
+          <t>東明-KY</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>356.6730637846136</v>
+        <v>374.2403813201082</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>35.8</v>
+        <v>32.45</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,13 +3520,13 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>41.90967229766305</v>
+        <v>43.37380752633383</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>23.56056004664616</v>
+        <v>32.84678507059154</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.1673063784613569</v>
+        <v>0.4240381320108234</v>
       </c>
       <c r="K58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.9582201256015994</v>
+        <v>-0.50265201916005</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>5907</v>
+        <v>4930</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>大洋-KY</t>
+          <t>燦星網</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>348.9084043967841</v>
+        <v>359.7198418646074</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>5.05</v>
+        <v>17.35</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,13 +3573,13 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>44.43552465861959</v>
+        <v>43.7333892054443</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>24.46292482884273</v>
+        <v>34.25901702495012</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.390840439678415</v>
+        <v>0.4719841864607431</v>
       </c>
       <c r="K59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.019279633521072</v>
+        <v>0.0277719202176923</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>4439</v>
+        <v>4562</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>冠星-KY</t>
+          <t>穎漢</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>337.3136490250697</v>
+        <v>356.6730637846136</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>90.09999999999999</v>
+        <v>35.8</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,13 +3626,13 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>42.65481014856325</v>
+        <v>41.90967229766305</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>46.41719972313586</v>
+        <v>23.56056004664616</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>1.231364902506964</v>
+        <v>0.1673063784613569</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.1616945748844021</v>
+        <v>-0.9582201256015994</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>6143</v>
+        <v>5907</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>振曜</t>
+          <t>大洋-KY</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>334.2136402283606</v>
+        <v>348.9084043967841</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>90.7</v>
+        <v>5.05</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,13 +3679,13 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>39.23101420571027</v>
+        <v>44.43552465861959</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>26.2865273900439</v>
+        <v>24.46292482884273</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.4213640228360623</v>
+        <v>0.390840439678415</v>
       </c>
       <c r="K61" s="2" t="n">
         <v>0</v>
@@ -3697,31 +3697,31 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-1.173885316988266</v>
+        <v>0.019279633521072</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>4426</v>
+        <v>4439</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>利勤</t>
+          <t>冠星-KY</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>323.9195357366331</v>
+        <v>337.3136490250697</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>8.01</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,13 +3732,13 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>47.68984921352049</v>
+        <v>42.65481014856325</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>21.86685742146232</v>
+        <v>46.41719972313586</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.3919535736633125</v>
+        <v>1.231364902506964</v>
       </c>
       <c r="K62" s="2" t="n">
         <v>0</v>
@@ -3750,31 +3750,31 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.0176346679571385</v>
+        <v>-0.1616945748844021</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>4737</v>
+        <v>6143</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>華廣</t>
+          <t>振曜</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>309.8989310899742</v>
+        <v>334.2136402283606</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>54.9</v>
+        <v>90.7</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,13 +3785,13 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>41.8516616153643</v>
+        <v>39.23101420571027</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>25.60136555828307</v>
+        <v>26.2865273900439</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.4898931089974225</v>
+        <v>0.4213640228360623</v>
       </c>
       <c r="K63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.0302076607319334</v>
+        <v>-1.173885316988266</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>4581</v>
+        <v>4426</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>光隆精密-KY</t>
+          <t>利勤</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>292.4156195413309</v>
+        <v>323.9195357366331</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>49.65</v>
+        <v>8.01</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,13 +3838,13 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>51.65028856950888</v>
+        <v>47.68984921352049</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>25.11037560195356</v>
+        <v>21.86685742146232</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>1.241561954133093</v>
+        <v>0.3919535736633125</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.5143923587615937</v>
+        <v>0.0176346679571385</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>4755</v>
+        <v>4737</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>三福化</t>
+          <t>華廣</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>291.6719102960272</v>
+        <v>309.8989310899742</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>140</v>
+        <v>54.9</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,13 +3891,13 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>45.61759100969651</v>
+        <v>41.8516616153643</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>18.36591962028105</v>
+        <v>25.60136555828307</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.6671910296027268</v>
+        <v>0.4898931089974225</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>0</v>
@@ -3909,31 +3909,31 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-1.387614401314258</v>
+        <v>0.0302076607319334</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>5521</v>
+        <v>4581</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>工信</t>
+          <t>光隆精密-KY</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>287.2582142974125</v>
+        <v>292.4156195413309</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>10.55</v>
+        <v>49.65</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,13 +3944,13 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>47.05597778740637</v>
+        <v>51.65028856950888</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>27.34548898249981</v>
+        <v>25.11037560195356</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>1.225821429741244</v>
+        <v>1.241561954133093</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.1236454581342041</v>
+        <v>0.5143923587615937</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>above_ema60, market_above_ma60, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>4560</v>
+        <v>4755</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>強信-KY</t>
+          <t>三福化</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>285.0919122674075</v>
+        <v>291.6719102960272</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>32.55</v>
+        <v>140</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,13 +3997,13 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>46.26830378037008</v>
+        <v>45.61759100969651</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>18.25026302152018</v>
+        <v>18.36591962028105</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>1.009191226740745</v>
+        <v>0.6671910296027268</v>
       </c>
       <c r="K67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.0544025902947936</v>
+        <v>-1.387614401314258</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>4195</v>
+        <v>5521</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>基米-創</t>
+          <t>工信</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>260.673408466547</v>
+        <v>287.2582142974125</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>16.3</v>
+        <v>10.55</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,13 +4050,13 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>26.88019506963234</v>
+        <v>47.05597778740637</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>45.2260666595232</v>
+        <v>27.34548898249981</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.5673408466546973</v>
+        <v>1.225821429741244</v>
       </c>
       <c r="K68" s="2" t="n">
         <v>0</v>
@@ -4068,31 +4068,31 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.2831333050658653</v>
+        <v>0.1236454581342041</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>5906</v>
+        <v>4560</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>台南-KY</t>
+          <t>強信-KY</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>255</v>
+        <v>285.0919122674075</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>0</v>
+        <v>32.55</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,13 +4103,13 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>46.04470615296958</v>
+        <v>46.26830378037008</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>7.91364784163176</v>
+        <v>18.25026302152018</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0</v>
+        <v>1.009191226740745</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>0</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-1.849094838025186</v>
+        <v>0.0544025902947936</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4131,21 +4131,21 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>4564</v>
+        <v>4195</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>元翎</t>
+          <t>基米-創</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>250.6963381814243</v>
+        <v>260.673408466547</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>15.45</v>
+        <v>16.3</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,13 +4156,13 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>37.83417426734455</v>
+        <v>26.88019506963234</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>38.6958056533116</v>
+        <v>45.2260666595232</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.5696338181424268</v>
+        <v>0.5673408466546973</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.06597526466791299</v>
+        <v>0.2831333050658653</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>4736</v>
+        <v>5906</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>泰博</t>
+          <t>台南-KY</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>221.8642497192834</v>
+        <v>255</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>124.5</v>
+        <v>0</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,13 +4209,13 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>50.61204993260861</v>
+        <v>46.04470615296958</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>12.50085462856218</v>
+        <v>7.91364784163176</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.6864249719283386</v>
+        <v>0</v>
       </c>
       <c r="K71" s="2" t="n">
         <v>0</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.1974116866264246</v>
+        <v>-1.849094838025186</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4237,21 +4237,21 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>4569</v>
+        <v>4564</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>六方科-KY</t>
+          <t>元翎</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>197.8100968716587</v>
+        <v>250.6963381814243</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>167.5</v>
+        <v>15.45</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,13 +4262,13 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>46.12657809803279</v>
+        <v>37.83417426734455</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>16.74161803794673</v>
+        <v>38.6958056533116</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.7810096871658698</v>
+        <v>0.5696338181424268</v>
       </c>
       <c r="K72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-1.670990161110644</v>
+        <v>0.06597526466791299</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>4746</v>
+        <v>4736</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>台耀</t>
+          <t>泰博</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>175.2351537526606</v>
+        <v>221.8642497192833</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>51.5</v>
+        <v>124.5</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,13 +4315,13 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>44.64154034557406</v>
+        <v>50.61204993260861</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>9.486846813901066</v>
+        <v>12.50085462856218</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>0.5235153752660638</v>
+        <v>0.6864249719283386</v>
       </c>
       <c r="K73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.0243230316248074</v>
+        <v>0.1974116866264246</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>5007</v>
+        <v>4569</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>三星</t>
+          <t>六方科-KY</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>172.7274487114792</v>
+        <v>197.8100968716587</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>56.5</v>
+        <v>167.5</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>45.30253361046012</v>
+        <v>46.12657809803279</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>19.28948318410757</v>
+        <v>16.74161803794673</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.2727448711479232</v>
+        <v>0.7810096871658698</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>0</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-0.1012909274172315</v>
+        <v>-1.670990161110644</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4396,21 +4396,21 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>6158</v>
+        <v>4746</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>禾昌</t>
+          <t>台耀</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>166.9668411193295</v>
+        <v>175.2351537526606</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>17.45</v>
+        <v>51.5</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,13 +4421,13 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>34.14393374638051</v>
+        <v>44.64154034557406</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>13.58761649835379</v>
+        <v>9.486846813901066</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>1.696684111932948</v>
+        <v>0.5235153752660638</v>
       </c>
       <c r="K75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-0.0188410825470713</v>
+        <v>-0.0243230316248074</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>4557</v>
+        <v>5007</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>永新-KY</t>
+          <t>三星</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>166.4967820064115</v>
+        <v>172.7274487114792</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>46.75</v>
+        <v>56.5</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,13 +4474,13 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>48.43621242024396</v>
+        <v>45.30253361046012</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>27.22166125974199</v>
+        <v>19.28948318410757</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.6496782006411473</v>
+        <v>0.2727448711479232</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.554729176980004</v>
+        <v>-0.1012909274172315</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>5546</v>
+        <v>6158</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>永固-KY</t>
+          <t>禾昌</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>148.8082868321468</v>
+        <v>166.9668411193295</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>16.75</v>
+        <v>17.45</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,13 +4527,13 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>50.81536816498284</v>
+        <v>34.14393374638051</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>23.09248744234548</v>
+        <v>13.58761649835379</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.3808286832146751</v>
+        <v>1.696684111932948</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.0242443830419427</v>
+        <v>-0.0188410825470713</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>4441</v>
+        <v>4557</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>振大環球</t>
+          <t>永新-KY</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>143.8922409045892</v>
+        <v>166.4967820064115</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>193.5</v>
+        <v>46.75</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,13 +4580,13 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>42.14477763333788</v>
+        <v>48.43621242024396</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>17.97233820215637</v>
+        <v>27.22166125974199</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.389224090458924</v>
+        <v>0.6496782006411473</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>0</v>
@@ -4598,31 +4598,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-2.115490011180428</v>
+        <v>0.554729176980004</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>4440</v>
+        <v>5546</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>宜新實業</t>
+          <t>永固-KY</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>124.4567220321029</v>
+        <v>148.8082868321468</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>17.15</v>
+        <v>16.75</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,13 +4633,13 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>37.99893325828462</v>
+        <v>50.81536816498284</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>16.63463066133024</v>
+        <v>23.09248744234548</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.4456722032102861</v>
+        <v>0.3808286832146751</v>
       </c>
       <c r="K79" s="2" t="n">
         <v>0</v>
@@ -4651,62 +4651,168 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.1217247489635101</v>
+        <v>0.0242443830419427</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
+        <v>4441</v>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>振大環球</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>143.8922409045892</v>
+      </c>
+      <c r="E80" s="2" t="n">
+        <v>193.5</v>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H80" s="2" t="n">
+        <v>42.14477763333788</v>
+      </c>
+      <c r="I80" s="2" t="n">
+        <v>17.97233820215637</v>
+      </c>
+      <c r="J80" s="2" t="n">
+        <v>0.389224090458924</v>
+      </c>
+      <c r="K80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N80" s="2" t="n">
+        <v>-2.115490011180428</v>
+      </c>
+      <c r="O80" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>4440</v>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>宜新實業</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>124.4567220321029</v>
+      </c>
+      <c r="E81" s="2" t="n">
+        <v>17.15</v>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H81" s="2" t="n">
+        <v>37.99893325828462</v>
+      </c>
+      <c r="I81" s="2" t="n">
+        <v>16.63463066133024</v>
+      </c>
+      <c r="J81" s="2" t="n">
+        <v>0.4456722032102861</v>
+      </c>
+      <c r="K81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M81" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N81" s="2" t="n">
+        <v>-0.1217247489635101</v>
+      </c>
+      <c r="O81" s="2" t="inlineStr">
+        <is>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
         <v>4770</v>
       </c>
-      <c r="B80" s="2" t="inlineStr">
+      <c r="B82" s="2" t="inlineStr">
         <is>
           <t>上品</t>
         </is>
       </c>
-      <c r="C80" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D80" s="2" t="n">
+      <c r="C82" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D82" s="2" t="n">
         <v>123.9487978910787</v>
       </c>
-      <c r="E80" s="2" t="n">
+      <c r="E82" s="2" t="n">
         <v>213.5</v>
       </c>
-      <c r="F80" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="G80" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H80" s="2" t="n">
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H82" s="2" t="n">
         <v>35.14166795768833</v>
       </c>
-      <c r="I80" s="2" t="n">
+      <c r="I82" s="2" t="n">
         <v>18.97149326314445</v>
       </c>
-      <c r="J80" s="2" t="n">
+      <c r="J82" s="2" t="n">
         <v>0.3948797891078702</v>
       </c>
-      <c r="K80" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L80" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M80" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N80" s="2" t="n">
+      <c r="K82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M82" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N82" s="2" t="n">
         <v>-4.525715643062574</v>
       </c>
-      <c r="O80" s="2" t="inlineStr">
+      <c r="O82" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>

</xml_diff>